<commit_message>
add types to workflow components
</commit_message>
<xml_diff>
--- a/workflows/csmWorkflow/isa.workflow.xlsx
+++ b/workflows/csmWorkflow/isa.workflow.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
   <si>
     <t>WORKFLOW</t>
   </si>
@@ -70,22 +70,43 @@
     <t>Workflow Parameters Name</t>
   </si>
   <si>
+    <t>crop modelling;simulation models</t>
+  </si>
+  <si>
     <t>Workflow Parameters Term Accession Number</t>
   </si>
   <si>
+    <t>C:9000024;C:24242</t>
+  </si>
+  <si>
     <t>Workflow Parameters Term Source REF</t>
   </si>
   <si>
+    <t>C;C</t>
+  </si>
+  <si>
     <t>Workflow Components Name</t>
   </si>
   <si>
+    <t>Docker image (EDAM:3973);DSSAT</t>
+  </si>
+  <si>
     <t>Workflow Components Type</t>
   </si>
   <si>
+    <t>Docker image;Simulation Files</t>
+  </si>
+  <si>
     <t>Workflow Components Type Term Accession Number</t>
   </si>
   <si>
+    <t>EDAM:3973;</t>
+  </si>
+  <si>
     <t>Workflow Components Type Term Source REF</t>
+  </si>
+  <si>
+    <t>edam;</t>
   </si>
   <si>
     <t>Workflow File Name</t>
@@ -589,142 +610,163 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="B12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+      <c r="B13" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+      <c r="B14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+      <c r="B15" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="B16" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>24</v>
+        <v>30</v>
+      </c>
+      <c r="B17" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="B18" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="B20" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="B21" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="B23" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="B24" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="B26" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="B27" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="B28" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="B29" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="B30" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="B31" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>